<commit_message>
Aktualizacja projektu zalecenia Zasady oceny ofert
</commit_message>
<xml_diff>
--- a/documentation/docs/zaopatrzenie/zasady-oceny-ofert/zasady-oceny-ofert-macierz-punktacji.xlsx
+++ b/documentation/docs/zaopatrzenie/zasady-oceny-ofert/zasady-oceny-ofert-macierz-punktacji.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\sdc\zaopatrzenie\01-zasady-oceny-ofert\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\siec-full\sdc\documentation\docs\zaopatrzenie\zasady-oceny-ofert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C819C3B0-6130-4F42-8BE2-6E45E0E78C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5C04B9-80AD-4CE0-B7E6-ED9FF3E46177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5ABF7374-C7EB-4C5D-B504-DEB8A40B4FFD}"/>
   </bookViews>
@@ -53,7 +53,7 @@
     Wg mnie punktacja W-01, W-02, W-06 i W-08 jest dobra</t>
       </text>
     </comment>
-    <comment ref="A7" authorId="1" shapeId="0" xr:uid="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
+    <comment ref="A8" authorId="1" shapeId="0" xr:uid="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -61,7 +61,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</t>
       </text>
     </comment>
-    <comment ref="A8" authorId="2" shapeId="0" xr:uid="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
+    <comment ref="A9" authorId="2" shapeId="0" xr:uid="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -69,7 +69,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi.</t>
       </text>
     </comment>
-    <comment ref="A9" authorId="3" shapeId="0" xr:uid="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
+    <comment ref="A10" authorId="3" shapeId="0" xr:uid="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -77,7 +77,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</t>
       </text>
     </comment>
-    <comment ref="A11" authorId="4" shapeId="0" xr:uid="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
+    <comment ref="A12" authorId="4" shapeId="0" xr:uid="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="85">
   <si>
     <t xml:space="preserve">Ocena ofert dostawy dostępnych rozwiązań cyfrowych 
 Szablon macierzy punktacji </t>
@@ -475,9 +475,6 @@
     </r>
   </si>
   <si>
-    <t>W-02</t>
-  </si>
-  <si>
     <t>Dostosowanie</t>
   </si>
   <si>
@@ -631,9 +628,6 @@
   </si>
   <si>
     <t>W-03</t>
-  </si>
-  <si>
-    <t>Tworzenie terści</t>
   </si>
   <si>
     <r>
@@ -1077,9 +1071,6 @@
   </si>
   <si>
     <t>W-07</t>
-  </si>
-  <si>
-    <t>Wskazówki</t>
   </si>
   <si>
     <r>
@@ -1667,10 +1658,6 @@
     </r>
   </si>
   <si>
-    <t>Ostatnia zmiana 
-20 września 2025</t>
-  </si>
-  <si>
     <t>wersja 1.0</t>
   </si>
   <si>
@@ -1713,13 +1700,699 @@
 PAD - Polski Akt dostępnmości (Ustawa o zapewnianiu spełniania wymagań dostępności niektórych produktów i usług przez podmioty gospodarcze)
 WCAG - Wytyczne dla dostępności treści internetowych </t>
     </r>
+  </si>
+  <si>
+    <t>W02</t>
+  </si>
+  <si>
+    <t>Wymagania dodatkowe</t>
+  </si>
+  <si>
+    <t>Tworzenie treści</t>
+  </si>
+  <si>
+    <t>W-08. Wskazówki dla użytkowników technologii wspomagających</t>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca opisuje sposób spełnienia wymagań dodatkowych oraz przedstawia częściowe dowody ich spełnienia lub plan ich realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przedstawia przykłady wcześniejszych wdrożeń spełniających podobne wymagania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca przedstawia kompleksowy opis sposobu spełnienia wszystkich wymagań dodatkowych wraz z odpowiednimi dowodami zgodności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca przedstawia wyniki testów, raporty lub inne materiały potwierdzające spełnienie wymagań wykraczających poza EN 301 549.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje możliwość spełnienia wymagań dodatkowych, ale nie przedstawia dowodów ani szczegółowego opisu sposobu ich realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca odnosi się tylko do części wymagań dodatkowych.</t>
+    </r>
+  </si>
+  <si>
+    <t>W-09</t>
+  </si>
+  <si>
+    <t>W-10</t>
+  </si>
+  <si>
+    <t>Komponenty stron trzecich</t>
+  </si>
+  <si>
+    <t>W-11</t>
+  </si>
+  <si>
+    <t>Utrzymanie dostępności</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze sposób utrzymywania dostępności rozwiązania po wdrożeniu, w tym proces zgłaszania, analizowania i usuwania problemów dostępności cyfrowej oraz sposób informowania nabywcy o zmianach mających wpływ na dostępność rozwiązania. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Dostawca określi sposób monitorowania dostępności rozwiązania, obsługi zgłoszeń dotyczących problemów dostępności oraz utrzymywania zgodności podczas aktualizacji, rozwoju i utrzymania rozwiązania. 
+Na przykład dostawca może przedstawić procedurę obsługi zgłoszeń, deklarowane czasy reakcji i usuwania błędów dostępności, sposób dokumentowania zmian wpływających na dostępność oraz zakres testów wykonywanych przed wdrożeniem nowych wersji rozwiązania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przedstawia dokumentację dostępności dla części komponentów stron trzecich oraz opisuje sposób monitorowania związanych z nimi ryzyk.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca wskazuje alternatywne rozwiązania lub działania ograniczające wpływ znanych problemów dostępności.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca opisuje proces zgłaszania, analizowania i usuwania problemów dostępności oraz sposób informowania nabywcy o postępie prac.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje wykonywanie testów dostępności przed wdrażaniem aktualizacji, ale nie przedstawia szczegółowych procedur lub mierników skuteczności.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca identyfikuje komponenty stron trzecich, ale przedstawia jedynie ogólne deklaracje dotyczące ich dostępności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie posiada dokumentacji dostępności komponentów, ale deklaruje możliwość jej pozyskania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca przedstawia dokumentację dostępności wszystkich kluczowych komponentów i usług stron trzecich oraz opisuje proces zarządzania ich dostępnością.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca posiada procedury monitorowania zmian, aktualizacji i zgłoszeń dotyczących dostępności komponentów stron trzecich oraz sposób reagowania na stwierdzone problemy.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze dostępność komponentów i usług stron trzecich stanowiących część oferowanego rozwiązania oraz sposób zarządzania ryzykiem związanym z ich dostępnością. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Dostawca określi, które elementy rozwiązania są dostarczane przez podmioty trzecie, jaki jest ich wpływ na dostępność całego rozwiązania oraz jakie informacje lub dowody dostępności są dostępne dla tych komponentów.
+Na przykład mogą to być moduły płatności elektronicznych, podpisu elektronicznego, map, komunikacji wideo, systemów uwierzytelniania, usług chmurowych lub innych usług integrowanych z rozwiązaniem. Dostawca powinien również opisać sposób postępowania w przypadku stwierdzenia problemów dostępności takich komponentów.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie identyfikuje komponentów lub usług stron trzecich wykorzystywanych w rozwiązaniu.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie posiada informacji dotyczących dostępności kluczowych komponentów stron trzecich.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca potwierdza istnienie znanych problemów dostępności komponentów stron trzecich bez planu ich ograniczania lub obejścia.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze sposób spełnienia dodatkowych wymagań dostępności określonych w dokumentacji zamówienia oraz przedstawi informacje lub dowody potwierdzające możliwość ich spełnienia. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Na przykład może to dotyczyć wybranych kryteriów sukcesu WCAG na poziomie AAA, dodatkowych wymagań dotyczących personalizacji interfejsu użytkownika, rozszerzonego wsparcia technologii wspomagających, wymagań wynikających ze specyfiki usługi lub szczególnych potrzeb użytkowników.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dokumentacja zamówienia zawiera dodatkowe wymagania dostępności, ale dostawca nie odniósł się do nich lub potwierdził, że nie planuje ich spełnić.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca ograniczył się do deklaracji zgodności z EN 301 549 bez przedstawienia informacji dotyczących wymagań dodatkowych.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca posiada udokumentowany proces utrzymywania dostępności obejmujący monitorowanie, zgłaszanie, analizowanie, usuwanie i weryfikację problemów dostępności.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca określa terminy reakcji i usuwania błędów dostępności, wykonuje testy dostępności przed publikacją nowych wersji oraz informuje nabywcę o zmianach mogących wpływać na dostępność rozwiązania.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca przedstawia dowody stosowania takiego procesu w innych wdrożeniach lub istniejących produktach.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje możliwość usuwania problemów dostępności, ale nie określa procesu, odpowiedzialności ani terminów realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przewiduje reakcję na zgłoszenia wyłącznie w ramach ogólnego procesu utrzymania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie opisuje sposobu utrzymywania dostępności po wdrożeniu.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie przewiduje procesu zgłaszania i usuwania problemów dostępności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca nie deklaruje działań związanych z testowaniem dostępności po aktualizacjach.</t>
+    </r>
+  </si>
+  <si>
+    <t>Ostatnia zmiana 
+24 czerwca 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1813,6 +2486,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1861,7 +2574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1929,6 +2642,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -2107,8 +2835,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}" name="Table2" displayName="Table2" ref="A4:G13" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A4:G13" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}" name="Table2" displayName="Table2" ref="A4:G16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A4:G16" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B6C24592-B29B-4A7A-92E7-3C12CB92CB2B}" name="Wymaganie" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{27A519DD-0FCC-40C2-8E6E-80209101DE7C}" name="Nazwa" dataDxfId="5"/>
@@ -2442,16 +3170,16 @@
   <threadedComment ref="A5" dT="2025-06-13T09:11:55.20" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{FA4ACAF5-889C-4668-8579-C7A217D5A1CA}">
     <text>Wg mnie punktacja W-01, W-02, W-06 i W-08 jest dobra</text>
   </threadedComment>
-  <threadedComment ref="A7" dT="2025-06-13T09:05:36.46" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
+  <threadedComment ref="A8" dT="2025-06-13T09:05:36.46" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
-  <threadedComment ref="A8" dT="2025-06-13T09:04:51.32" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
+  <threadedComment ref="A9" dT="2025-06-13T09:04:51.32" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi.</text>
   </threadedComment>
-  <threadedComment ref="A9" dT="2025-06-13T09:05:43.82" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
+  <threadedComment ref="A10" dT="2025-06-13T09:05:43.82" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
-  <threadedComment ref="A11" dT="2025-06-13T09:05:51.24" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
+  <threadedComment ref="A12" dT="2025-06-13T09:05:51.24" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
 </ThreadedComments>
@@ -2459,11 +3187,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{885FD296-1036-4B63-BFFE-0A02F1DC228A}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="72.44140625" style="1" customWidth="1"/>
     <col min="4" max="7" width="67.109375" style="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="1"/>
@@ -2482,7 +3210,7 @@
     </row>
     <row r="2" spans="1:7" ht="192.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -2493,10 +3221,10 @@
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -2535,7 +3263,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>10</v>
@@ -2550,177 +3278,246 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="206.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="243" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="206.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C7" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="276" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="184.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="D10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="7" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="15" t="s">
+    <row r="11" spans="1:7" ht="211.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>25</v>
+      <c r="D11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="276" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="15" t="s">
+    <row r="12" spans="1:7" ht="202.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>19</v>
+      <c r="D12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="184.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="15" t="s">
+    <row r="13" spans="1:7" ht="266.39999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>19</v>
+      <c r="D13" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="211.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>19</v>
+    <row r="14" spans="1:7" ht="346.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="202.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>46</v>
+    <row r="15" spans="1:7" ht="266.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D12" s="11" t="s">
+    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2875,18 +3672,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2908,14 +3705,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{196F5893-5B18-4A2E-91AB-1824D20461F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{595289A5-1413-4EA3-A6CA-9B9CCFA1C57D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -2929,4 +3718,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{196F5893-5B18-4A2E-91AB-1824D20461F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Usunięcie zmian spoza zakresu kontroli przed publikacją
</commit_message>
<xml_diff>
--- a/documentation/docs/zaopatrzenie/zasady-oceny-ofert/zasady-oceny-ofert-macierz-punktacji.xlsx
+++ b/documentation/docs/zaopatrzenie/zasady-oceny-ofert/zasady-oceny-ofert-macierz-punktacji.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\sdc\zaopatrzenie\01-zasady-oceny-ofert\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\siec-full\sdc\documentation\docs\zaopatrzenie\zasady-oceny-ofert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C819C3B0-6130-4F42-8BE2-6E45E0E78C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5C04B9-80AD-4CE0-B7E6-ED9FF3E46177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5ABF7374-C7EB-4C5D-B504-DEB8A40B4FFD}"/>
   </bookViews>
@@ -53,7 +53,7 @@
     Wg mnie punktacja W-01, W-02, W-06 i W-08 jest dobra</t>
       </text>
     </comment>
-    <comment ref="A7" authorId="1" shapeId="0" xr:uid="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
+    <comment ref="A8" authorId="1" shapeId="0" xr:uid="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -61,7 +61,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</t>
       </text>
     </comment>
-    <comment ref="A8" authorId="2" shapeId="0" xr:uid="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
+    <comment ref="A9" authorId="2" shapeId="0" xr:uid="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -69,7 +69,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi.</t>
       </text>
     </comment>
-    <comment ref="A9" authorId="3" shapeId="0" xr:uid="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
+    <comment ref="A10" authorId="3" shapeId="0" xr:uid="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -77,7 +77,7 @@
     Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</t>
       </text>
     </comment>
-    <comment ref="A11" authorId="4" shapeId="0" xr:uid="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
+    <comment ref="A12" authorId="4" shapeId="0" xr:uid="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
       <text>
         <t>[Komentarz podzielony na wątki]
 Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="85">
   <si>
     <t xml:space="preserve">Ocena ofert dostawy dostępnych rozwiązań cyfrowych 
 Szablon macierzy punktacji </t>
@@ -475,9 +475,6 @@
     </r>
   </si>
   <si>
-    <t>W-02</t>
-  </si>
-  <si>
     <t>Dostosowanie</t>
   </si>
   <si>
@@ -631,9 +628,6 @@
   </si>
   <si>
     <t>W-03</t>
-  </si>
-  <si>
-    <t>Tworzenie terści</t>
   </si>
   <si>
     <r>
@@ -1077,9 +1071,6 @@
   </si>
   <si>
     <t>W-07</t>
-  </si>
-  <si>
-    <t>Wskazówki</t>
   </si>
   <si>
     <r>
@@ -1667,10 +1658,6 @@
     </r>
   </si>
   <si>
-    <t>Ostatnia zmiana 
-20 września 2025</t>
-  </si>
-  <si>
     <t>wersja 1.0</t>
   </si>
   <si>
@@ -1713,13 +1700,699 @@
 PAD - Polski Akt dostępnmości (Ustawa o zapewnianiu spełniania wymagań dostępności niektórych produktów i usług przez podmioty gospodarcze)
 WCAG - Wytyczne dla dostępności treści internetowych </t>
     </r>
+  </si>
+  <si>
+    <t>W02</t>
+  </si>
+  <si>
+    <t>Wymagania dodatkowe</t>
+  </si>
+  <si>
+    <t>Tworzenie treści</t>
+  </si>
+  <si>
+    <t>W-08. Wskazówki dla użytkowników technologii wspomagających</t>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca opisuje sposób spełnienia wymagań dodatkowych oraz przedstawia częściowe dowody ich spełnienia lub plan ich realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przedstawia przykłady wcześniejszych wdrożeń spełniających podobne wymagania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca przedstawia kompleksowy opis sposobu spełnienia wszystkich wymagań dodatkowych wraz z odpowiednimi dowodami zgodności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca przedstawia wyniki testów, raporty lub inne materiały potwierdzające spełnienie wymagań wykraczających poza EN 301 549.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje możliwość spełnienia wymagań dodatkowych, ale nie przedstawia dowodów ani szczegółowego opisu sposobu ich realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca odnosi się tylko do części wymagań dodatkowych.</t>
+    </r>
+  </si>
+  <si>
+    <t>W-09</t>
+  </si>
+  <si>
+    <t>W-10</t>
+  </si>
+  <si>
+    <t>Komponenty stron trzecich</t>
+  </si>
+  <si>
+    <t>W-11</t>
+  </si>
+  <si>
+    <t>Utrzymanie dostępności</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze sposób utrzymywania dostępności rozwiązania po wdrożeniu, w tym proces zgłaszania, analizowania i usuwania problemów dostępności cyfrowej oraz sposób informowania nabywcy o zmianach mających wpływ na dostępność rozwiązania. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Dostawca określi sposób monitorowania dostępności rozwiązania, obsługi zgłoszeń dotyczących problemów dostępności oraz utrzymywania zgodności podczas aktualizacji, rozwoju i utrzymania rozwiązania. 
+Na przykład dostawca może przedstawić procedurę obsługi zgłoszeń, deklarowane czasy reakcji i usuwania błędów dostępności, sposób dokumentowania zmian wpływających na dostępność oraz zakres testów wykonywanych przed wdrożeniem nowych wersji rozwiązania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przedstawia dokumentację dostępności dla części komponentów stron trzecich oraz opisuje sposób monitorowania związanych z nimi ryzyk.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca wskazuje alternatywne rozwiązania lub działania ograniczające wpływ znanych problemów dostępności.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca opisuje proces zgłaszania, analizowania i usuwania problemów dostępności oraz sposób informowania nabywcy o postępie prac.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje wykonywanie testów dostępności przed wdrażaniem aktualizacji, ale nie przedstawia szczegółowych procedur lub mierników skuteczności.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca identyfikuje komponenty stron trzecich, ale przedstawia jedynie ogólne deklaracje dotyczące ich dostępności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie posiada dokumentacji dostępności komponentów, ale deklaruje możliwość jej pozyskania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca przedstawia dokumentację dostępności wszystkich kluczowych komponentów i usług stron trzecich oraz opisuje proces zarządzania ich dostępnością.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca posiada procedury monitorowania zmian, aktualizacji i zgłoszeń dotyczących dostępności komponentów stron trzecich oraz sposób reagowania na stwierdzone problemy.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze dostępność komponentów i usług stron trzecich stanowiących część oferowanego rozwiązania oraz sposób zarządzania ryzykiem związanym z ich dostępnością. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Dostawca określi, które elementy rozwiązania są dostarczane przez podmioty trzecie, jaki jest ich wpływ na dostępność całego rozwiązania oraz jakie informacje lub dowody dostępności są dostępne dla tych komponentów.
+Na przykład mogą to być moduły płatności elektronicznych, podpisu elektronicznego, map, komunikacji wideo, systemów uwierzytelniania, usług chmurowych lub innych usług integrowanych z rozwiązaniem. Dostawca powinien również opisać sposób postępowania w przypadku stwierdzenia problemów dostępności takich komponentów.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie identyfikuje komponentów lub usług stron trzecich wykorzystywanych w rozwiązaniu.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie posiada informacji dotyczących dostępności kluczowych komponentów stron trzecich.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca potwierdza istnienie znanych problemów dostępności komponentów stron trzecich bez planu ich ograniczania lub obejścia.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">Dostawca opisze sposób spełnienia dodatkowych wymagań dostępności określonych w dokumentacji zamówienia oraz przedstawi informacje lub dowody potwierdzające możliwość ich spełnienia. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Na przykład może to dotyczyć wybranych kryteriów sukcesu WCAG na poziomie AAA, dodatkowych wymagań dotyczących personalizacji interfejsu użytkownika, rozszerzonego wsparcia technologii wspomagających, wymagań wynikających ze specyfiki usługi lub szczególnych potrzeb użytkowników.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dokumentacja zamówienia zawiera dodatkowe wymagania dostępności, ale dostawca nie odniósł się do nich lub potwierdził, że nie planuje ich spełnić.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca ograniczył się do deklaracji zgodności z EN 301 549 bez przedstawienia informacji dotyczących wymagań dodatkowych.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca posiada udokumentowany proces utrzymywania dostępności obejmujący monitorowanie, zgłaszanie, analizowanie, usuwanie i weryfikację problemów dostępności.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca określa terminy reakcji i usuwania błędów dostępności, wykonuje testy dostępności przed publikacją nowych wersji oraz informuje nabywcę o zmianach mogących wpływać na dostępność rozwiązania.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+(Dowolne) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dostawca przedstawia dowody stosowania takiego procesu w innych wdrożeniach lub istniejących produktach.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca deklaruje możliwość usuwania problemów dostępności, ale nie określa procesu, odpowiedzialności ani terminów realizacji.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca przewiduje reakcję na zgłoszenia wyłącznie w ramach ogólnego procesu utrzymania.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie opisuje sposobu utrzymywania dostępności po wdrożeniu.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Dostawca nie przewiduje procesu zgłaszania i usuwania problemów dostępności.
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Dowolne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>) Dostawca nie deklaruje działań związanych z testowaniem dostępności po aktualizacjach.</t>
+    </r>
+  </si>
+  <si>
+    <t>Ostatnia zmiana 
+24 czerwca 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1813,6 +2486,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1861,7 +2574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1929,6 +2642,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -2107,8 +2835,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}" name="Table2" displayName="Table2" ref="A4:G13" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A4:G13" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}" name="Table2" displayName="Table2" ref="A4:G16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A4:G16" xr:uid="{52F17FEA-42D0-4E6C-8B68-B87EDC108F6F}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B6C24592-B29B-4A7A-92E7-3C12CB92CB2B}" name="Wymaganie" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{27A519DD-0FCC-40C2-8E6E-80209101DE7C}" name="Nazwa" dataDxfId="5"/>
@@ -2442,16 +3170,16 @@
   <threadedComment ref="A5" dT="2025-06-13T09:11:55.20" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{FA4ACAF5-889C-4668-8579-C7A217D5A1CA}">
     <text>Wg mnie punktacja W-01, W-02, W-06 i W-08 jest dobra</text>
   </threadedComment>
-  <threadedComment ref="A7" dT="2025-06-13T09:05:36.46" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
+  <threadedComment ref="A8" dT="2025-06-13T09:05:36.46" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{63B857A1-6FBD-4CA9-BD91-8C1149D1A1AF}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
-  <threadedComment ref="A8" dT="2025-06-13T09:04:51.32" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
+  <threadedComment ref="A9" dT="2025-06-13T09:04:51.32" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{19121E6F-3BE7-458D-8D92-2C3DD43491A3}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi.</text>
   </threadedComment>
-  <threadedComment ref="A9" dT="2025-06-13T09:05:43.82" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
+  <threadedComment ref="A10" dT="2025-06-13T09:05:43.82" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{600828BB-2E2C-48EF-AB26-98F7FA0F7748}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
-  <threadedComment ref="A11" dT="2025-06-13T09:05:51.24" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
+  <threadedComment ref="A12" dT="2025-06-13T09:05:51.24" personId="{304D56E0-DECA-4423-A969-AABB31511B96}" id="{0FE4ABD7-6413-4BC8-AA42-61D14CAF5A6A}">
     <text>Do tych wymagań (W03, W04, W-05, W-07) w opisie dobrej praktyki dodałam komentarze, dlatego tu nie poświęcam im już uwagi</text>
   </threadedComment>
 </ThreadedComments>
@@ -2459,11 +3187,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{885FD296-1036-4B63-BFFE-0A02F1DC228A}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="72.44140625" style="1" customWidth="1"/>
     <col min="4" max="7" width="67.109375" style="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="1"/>
@@ -2482,7 +3210,7 @@
     </row>
     <row r="2" spans="1:7" ht="192.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -2493,10 +3221,10 @@
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -2535,7 +3263,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>10</v>
@@ -2550,177 +3278,246 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="206.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="243" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="206.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C7" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="276" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="184.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="D10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="7" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="15" t="s">
+    <row r="11" spans="1:7" ht="211.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>25</v>
+      <c r="D11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="276" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="15" t="s">
+    <row r="12" spans="1:7" ht="202.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>19</v>
+      <c r="D12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="184.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="15" t="s">
+    <row r="13" spans="1:7" ht="266.39999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>19</v>
+      <c r="D13" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="211.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>19</v>
+    <row r="14" spans="1:7" ht="346.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="202.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>46</v>
+    <row r="15" spans="1:7" ht="266.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D12" s="11" t="s">
+    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2875,18 +3672,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2908,14 +3705,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{196F5893-5B18-4A2E-91AB-1824D20461F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{595289A5-1413-4EA3-A6CA-9B9CCFA1C57D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -2929,4 +3718,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{196F5893-5B18-4A2E-91AB-1824D20461F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>